<commit_message>
Sync authoritative 8088 history through Event 72
</commit_message>
<xml_diff>
--- a/data/Barrister_Master.xlsx
+++ b/data/Barrister_Master.xlsx
@@ -904,10 +904,10 @@
         <v>Completed Service Events</v>
       </c>
       <c r="B2" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C2" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" ht="15" hidden="0" customHeight="1">
@@ -926,10 +926,10 @@
         <v>Total Timeline Positions</v>
       </c>
       <c r="B4" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C4" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="5" ht="15" hidden="0" customHeight="1">
@@ -937,10 +937,10 @@
         <v>Completed Unique Clients</v>
       </c>
       <c r="B5" s="15">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" s="15">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="6" ht="15" hidden="0" customHeight="1">
@@ -948,10 +948,10 @@
         <v>Forward-Looking Client Count</v>
       </c>
       <c r="B6" s="15">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C6" s="15">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="7" ht="15" hidden="0" customHeight="1">
@@ -1027,7 +1027,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J70"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="9" hidden="0" customWidth="1"/>
@@ -4150,7 +4150,7 @@
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Fallston</t>
+          <t>Aberdeen</t>
         </is>
       </c>
       <c r="G68" t="inlineStr">
@@ -4170,7 +4170,7 @@
       </c>
       <c r="J68" t="inlineStr">
         <is>
-          <t>Project</t>
+          <t>Part 2</t>
         </is>
       </c>
     </row>
@@ -4180,12 +4180,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>TJ Maxx</t>
+          <t>Dunkin</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Columbia</t>
+          <t>Fallston</t>
         </is>
       </c>
       <c r="G69" t="inlineStr">
@@ -4205,7 +4205,7 @@
       </c>
       <c r="J69" t="inlineStr">
         <is>
-          <t>TJX Project</t>
+          <t>Project</t>
         </is>
       </c>
     </row>
@@ -4215,27 +4215,137 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
+          <t>TJ Maxx</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Columbia</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>TJX</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71">
+        <v>70</v>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
           <t>Giant Food Stores</t>
         </is>
       </c>
-      <c r="F70" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>Olney</t>
         </is>
       </c>
-      <c r="G70" t="inlineStr">
+      <c r="G71" t="inlineStr">
         <is>
           <t>MD</t>
         </is>
       </c>
-      <c r="H70" t="inlineStr">
+      <c r="H71" t="inlineStr">
         <is>
           <t>Maryland</t>
         </is>
       </c>
-      <c r="I70" t="inlineStr">
-        <is>
-          <t>Completed</t>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>Server</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72">
+        <v>71</v>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>WeWork</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>Washington</t>
+        </is>
+      </c>
+      <c r="G72" t="inlineStr">
+        <is>
+          <t>DC</t>
+        </is>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>Washington, D.C.</t>
+        </is>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>Server install</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73">
+        <v>72</v>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Hebrew Home of Greater Washington</t>
+        </is>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>North Bethesda</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>MD</t>
+        </is>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>Maryland</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>Printer</t>
         </is>
       </c>
     </row>
@@ -4285,7 +4395,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G54"/>
+  <dimension ref="A1:G55"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="10" hidden="0" customWidth="1"/>
@@ -5264,7 +5374,7 @@
         </is>
       </c>
       <c r="E32">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
@@ -5852,7 +5962,7 @@
         </is>
       </c>
       <c r="E53">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
@@ -5888,6 +5998,34 @@
         </is>
       </c>
       <c r="G54" t="inlineStr">
+        <is>
+          <t>Single</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>WeWork</t>
+        </is>
+      </c>
+      <c r="C55">
+        <v>71</v>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="E55">
+        <v>1</v>
+      </c>
+      <c r="F55" t="inlineStr">
+        <is>
+          <t>Completed</t>
+        </is>
+      </c>
+      <c r="G55" t="inlineStr">
         <is>
           <t>Single</t>
         </is>
@@ -5950,7 +6088,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>30, 34, 39, 61, 62, 66, 68</t>
+          <t>30, 34, 39, 61, 62, 66, 69</t>
         </is>
       </c>
     </row>
@@ -5972,7 +6110,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Marshalls</t>
+          <t>Dunkin</t>
         </is>
       </c>
       <c r="B4">
@@ -5980,44 +6118,44 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>35, 44, 46, 63, 64</t>
+          <t>56, 58, 59, 67, 68</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Dunkin</t>
+          <t>Hebrew Home of Greater Washington</t>
         </is>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>56, 58, 59, 67</t>
+          <t>8, 33, 48, 51, 72</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Giant Food Stores</t>
+          <t>Marshalls</t>
         </is>
       </c>
       <c r="B6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>10, 20, 50, 69</t>
+          <t>35, 44, 46, 63, 64</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Hebrew Home of Greater Washington</t>
+          <t>Giant Food Stores</t>
         </is>
       </c>
       <c r="B7">
@@ -6025,7 +6163,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>8, 33, 48, 51</t>
+          <t>10, 20, 50, 70</t>
         </is>
       </c>
     </row>
@@ -6272,13 +6410,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C2">
         <v>0</v>
       </c>
       <c r="D2">
-        <v>48</v>
+        <v>50</v>
       </c>
     </row>
     <row r="3">
@@ -6288,13 +6426,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="C3">
         <v>0</v>
       </c>
       <c r="D3">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="4">
@@ -6355,7 +6493,7 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="8" hidden="0" customWidth="1"/>
@@ -6665,6 +6803,33 @@
       <c r="F11" t="inlineStr">
         <is>
           <t>TJX Project</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Autumn Lake</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Glen Burnie, MD</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>2026-07-20</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Scheduled</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Printer</t>
         </is>
       </c>
     </row>
@@ -7026,10 +7191,10 @@
         <v>Completed Service Events</v>
       </c>
       <c r="B2" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C2" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="3" ht="15" hidden="0" customHeight="1">
@@ -7037,10 +7202,10 @@
         <v>Completed Unique Clients</v>
       </c>
       <c r="B3" s="15">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C3" s="15">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="4" ht="15" hidden="0" customHeight="1">
@@ -7048,10 +7213,10 @@
         <v>Forward-Looking Client Count</v>
       </c>
       <c r="B4" s="15">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="C4" s="15">
-        <v>53</v>
+        <v>54</v>
       </c>
     </row>
     <row r="5" ht="15" hidden="0" customHeight="1">
@@ -7059,10 +7224,10 @@
         <v>Timeline Max Position</v>
       </c>
       <c r="B5" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C5" s="15">
-        <v>69</v>
+        <v>72</v>
       </c>
     </row>
     <row r="6" ht="15" hidden="0" customHeight="1">

</xml_diff>